<commit_message>
LMDI: Merge pull request #78 from folkehelseinstituttet/fix/organisatorisk-betegnelse-short
Legg til short-beskrivelse for organisatoriskBetegnelse (#67) ff1a4af258e73f67cb5a745ecfbe183fbfa43bf9
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-lmdi-organization.xlsx
+++ b/currentbuild/StructureDefinition-lmdi-organization.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3220" uniqueCount="572">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3220" uniqueCount="573">
   <si>
     <t>Property</t>
   </si>
@@ -1108,7 +1108,10 @@
     <t>organisatoriskBetegnelse</t>
   </si>
   <si>
-    <t>Organisatorisk betegnelse</t>
+    <t>Organisatorisk betegnelse. Kodeverk "Organisatorisk betegnelse" (OID 8624)</t>
+  </si>
+  <si>
+    <t>Kode fra kodeverk "Organisatorisk betegnelse" (OID 8624) som beskriver type organisatorisk enhet (f.eks. sykehus, avdeling, klinikk)</t>
   </si>
   <si>
     <t>urn:oid:2.16.578.1.12.4.1.1.8624</t>
@@ -7136,7 +7139,7 @@
         <v>351</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>278</v>
+        <v>352</v>
       </c>
       <c r="N44" t="s" s="2">
         <v>266</v>
@@ -7171,7 +7174,7 @@
       </c>
       <c r="Y44" s="2"/>
       <c r="Z44" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="AA44" t="s" s="2">
         <v>77</v>
@@ -7218,7 +7221,7 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B45" t="s" s="2">
         <v>281</v>
@@ -7330,7 +7333,7 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B46" t="s" s="2">
         <v>283</v>
@@ -7444,7 +7447,7 @@
     </row>
     <row r="47" hidden="true">
       <c r="A47" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B47" t="s" s="2">
         <v>285</v>
@@ -7560,7 +7563,7 @@
     </row>
     <row r="48" hidden="true">
       <c r="A48" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B48" t="s" s="2">
         <v>295</v>
@@ -7672,7 +7675,7 @@
     </row>
     <row r="49" hidden="true">
       <c r="A49" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B49" t="s" s="2">
         <v>297</v>
@@ -7786,7 +7789,7 @@
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B50" t="s" s="2">
         <v>299</v>
@@ -7831,7 +7834,7 @@
       </c>
       <c r="Q50" s="2"/>
       <c r="R50" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="S50" t="s" s="2">
         <v>77</v>
@@ -7902,7 +7905,7 @@
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B51" t="s" s="2">
         <v>308</v>
@@ -8016,7 +8019,7 @@
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B52" t="s" s="2">
         <v>316</v>
@@ -8130,7 +8133,7 @@
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B53" t="s" s="2">
         <v>324</v>
@@ -8244,7 +8247,7 @@
     </row>
     <row r="54" hidden="true">
       <c r="A54" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B54" t="s" s="2">
         <v>332</v>
@@ -8360,7 +8363,7 @@
     </row>
     <row r="55" hidden="true">
       <c r="A55" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B55" t="s" s="2">
         <v>341</v>
@@ -8476,10 +8479,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8505,16 +8508,16 @@
         <v>164</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="N56" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="O56" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="P56" t="s" s="2">
         <v>77</v>
@@ -8563,7 +8566,7 @@
         <v>77</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>78</v>
@@ -8578,13 +8581,13 @@
         <v>99</v>
       </c>
       <c r="AK56" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="AL56" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="AM56" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="AN56" t="s" s="2">
         <v>77</v>
@@ -8592,10 +8595,10 @@
     </row>
     <row r="57" hidden="true">
       <c r="A57" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8621,16 +8624,16 @@
         <v>164</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="N57" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="O57" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="P57" t="s" s="2">
         <v>77</v>
@@ -8679,7 +8682,7 @@
         <v>77</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>78</v>
@@ -8697,7 +8700,7 @@
         <v>77</v>
       </c>
       <c r="AL57" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="AM57" t="s" s="2">
         <v>77</v>
@@ -8708,10 +8711,10 @@
     </row>
     <row r="58" hidden="true">
       <c r="A58" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -8734,19 +8737,19 @@
         <v>77</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="N58" t="s" s="2">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="O58" t="s" s="2">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="P58" t="s" s="2">
         <v>77</v>
@@ -8795,7 +8798,7 @@
         <v>77</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>78</v>
@@ -8804,19 +8807,19 @@
         <v>79</v>
       </c>
       <c r="AI58" t="s" s="2">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="AJ58" t="s" s="2">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="AK58" t="s" s="2">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="AL58" t="s" s="2">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="AM58" t="s" s="2">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="AN58" t="s" s="2">
         <v>77</v>
@@ -8824,10 +8827,10 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -8850,19 +8853,19 @@
         <v>77</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="N59" t="s" s="2">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="O59" t="s" s="2">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="P59" t="s" s="2">
         <v>77</v>
@@ -8911,7 +8914,7 @@
         <v>77</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>78</v>
@@ -8920,19 +8923,19 @@
         <v>79</v>
       </c>
       <c r="AI59" t="s" s="2">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="AJ59" t="s" s="2">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="AK59" t="s" s="2">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="AL59" t="s" s="2">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="AM59" t="s" s="2">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="AN59" t="s" s="2">
         <v>77</v>
@@ -8940,10 +8943,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -9052,10 +9055,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -9081,10 +9084,10 @@
         <v>133</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="N61" s="2"/>
       <c r="O61" s="2"/>
@@ -9164,13 +9167,13 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C62" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D62" t="s" s="2">
         <v>77</v>
@@ -9192,13 +9195,13 @@
         <v>77</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
@@ -9278,16 +9281,16 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C63" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D63" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E63" s="2"/>
       <c r="F63" t="s" s="2">
@@ -9306,13 +9309,13 @@
         <v>77</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="N63" s="2"/>
       <c r="O63" s="2"/>
@@ -9392,13 +9395,13 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C64" t="s" s="2">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D64" t="s" s="2">
         <v>77</v>
@@ -9420,13 +9423,13 @@
         <v>77</v>
       </c>
       <c r="K64" t="s" s="2">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="N64" s="2"/>
       <c r="O64" s="2"/>
@@ -9506,10 +9509,10 @@
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -9535,16 +9538,16 @@
         <v>107</v>
       </c>
       <c r="L65" t="s" s="2">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="M65" t="s" s="2">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="N65" t="s" s="2">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="O65" t="s" s="2">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="P65" t="s" s="2">
         <v>77</v>
@@ -9557,7 +9560,7 @@
         <v>77</v>
       </c>
       <c r="T65" t="s" s="2">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="U65" t="s" s="2">
         <v>77</v>
@@ -9572,10 +9575,10 @@
         <v>181</v>
       </c>
       <c r="Y65" t="s" s="2">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="Z65" t="s" s="2">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="AA65" t="s" s="2">
         <v>77</v>
@@ -9593,7 +9596,7 @@
         <v>77</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>78</v>
@@ -9608,13 +9611,13 @@
         <v>99</v>
       </c>
       <c r="AK65" t="s" s="2">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="AL65" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="AM65" t="s" s="2">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="AN65" t="s" s="2">
         <v>77</v>
@@ -9622,10 +9625,10 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -9651,13 +9654,13 @@
         <v>107</v>
       </c>
       <c r="L66" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="M66" t="s" s="2">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="N66" t="s" s="2">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="O66" s="2"/>
       <c r="P66" t="s" s="2">
@@ -9668,10 +9671,10 @@
         <v>77</v>
       </c>
       <c r="S66" t="s" s="2">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="T66" t="s" s="2">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="U66" t="s" s="2">
         <v>77</v>
@@ -9687,7 +9690,7 @@
       </c>
       <c r="Y66" s="2"/>
       <c r="Z66" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="AA66" t="s" s="2">
         <v>77</v>
@@ -9705,7 +9708,7 @@
         <v>77</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="AG66" t="s" s="2">
         <v>78</v>
@@ -9720,10 +9723,10 @@
         <v>99</v>
       </c>
       <c r="AK66" t="s" s="2">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="AL66" t="s" s="2">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="AM66" t="s" s="2">
         <v>77</v>
@@ -9734,10 +9737,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -9763,16 +9766,16 @@
         <v>164</v>
       </c>
       <c r="L67" t="s" s="2">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="M67" t="s" s="2">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="N67" t="s" s="2">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="O67" t="s" s="2">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="P67" t="s" s="2">
         <v>77</v>
@@ -9785,7 +9788,7 @@
         <v>77</v>
       </c>
       <c r="T67" t="s" s="2">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="U67" t="s" s="2">
         <v>77</v>
@@ -9821,7 +9824,7 @@
         <v>77</v>
       </c>
       <c r="AF67" t="s" s="2">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="AG67" t="s" s="2">
         <v>78</v>
@@ -9836,10 +9839,10 @@
         <v>99</v>
       </c>
       <c r="AK67" t="s" s="2">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="AL67" t="s" s="2">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="AM67" t="s" s="2">
         <v>77</v>
@@ -9850,10 +9853,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -9879,10 +9882,10 @@
         <v>164</v>
       </c>
       <c r="L68" t="s" s="2">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="M68" t="s" s="2">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
@@ -9897,7 +9900,7 @@
         <v>77</v>
       </c>
       <c r="T68" t="s" s="2">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="U68" t="s" s="2">
         <v>77</v>
@@ -9933,7 +9936,7 @@
         <v>77</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>78</v>
@@ -9948,13 +9951,13 @@
         <v>99</v>
       </c>
       <c r="AK68" t="s" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="AL68" t="s" s="2">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="AM68" t="s" s="2">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="AN68" t="s" s="2">
         <v>77</v>
@@ -9962,14 +9965,14 @@
     </row>
     <row r="69" hidden="true">
       <c r="A69" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="E69" s="2"/>
       <c r="F69" t="s" s="2">
@@ -9991,10 +9994,10 @@
         <v>164</v>
       </c>
       <c r="L69" t="s" s="2">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="M69" t="s" s="2">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="N69" s="2"/>
       <c r="O69" s="2"/>
@@ -10009,7 +10012,7 @@
         <v>77</v>
       </c>
       <c r="T69" t="s" s="2">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="U69" t="s" s="2">
         <v>77</v>
@@ -10045,7 +10048,7 @@
         <v>77</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>78</v>
@@ -10060,13 +10063,13 @@
         <v>99</v>
       </c>
       <c r="AK69" t="s" s="2">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="AL69" t="s" s="2">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="AM69" t="s" s="2">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="AN69" t="s" s="2">
         <v>77</v>
@@ -10074,14 +10077,14 @@
     </row>
     <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="E70" s="2"/>
       <c r="F70" t="s" s="2">
@@ -10103,13 +10106,13 @@
         <v>164</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="N70" t="s" s="2">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="O70" s="2"/>
       <c r="P70" t="s" s="2">
@@ -10123,7 +10126,7 @@
         <v>77</v>
       </c>
       <c r="T70" t="s" s="2">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="U70" t="s" s="2">
         <v>77</v>
@@ -10159,7 +10162,7 @@
         <v>77</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>78</v>
@@ -10174,10 +10177,10 @@
         <v>99</v>
       </c>
       <c r="AK70" t="s" s="2">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="AL70" t="s" s="2">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="AM70" t="s" s="2">
         <v>77</v>
@@ -10188,10 +10191,10 @@
     </row>
     <row r="71" hidden="true">
       <c r="A71" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -10217,10 +10220,10 @@
         <v>164</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
@@ -10300,10 +10303,10 @@
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -10329,10 +10332,10 @@
         <v>133</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="N72" s="2"/>
       <c r="O72" s="2"/>
@@ -10410,13 +10413,13 @@
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
+        <v>479</v>
+      </c>
+      <c r="B73" t="s" s="2">
         <v>478</v>
       </c>
-      <c r="B73" t="s" s="2">
-        <v>477</v>
-      </c>
       <c r="C73" t="s" s="2">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="D73" t="s" s="2">
         <v>77</v>
@@ -10438,13 +10441,13 @@
         <v>77</v>
       </c>
       <c r="K73" t="s" s="2">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="L73" t="s" s="2">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="M73" t="s" s="2">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="N73" s="2"/>
       <c r="O73" s="2"/>
@@ -10504,7 +10507,7 @@
         <v>79</v>
       </c>
       <c r="AI73" t="s" s="2">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="AJ73" t="s" s="2">
         <v>138</v>
@@ -10524,10 +10527,10 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -10553,10 +10556,10 @@
         <v>164</v>
       </c>
       <c r="L74" t="s" s="2">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="M74" t="s" s="2">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="N74" s="2"/>
       <c r="O74" s="2"/>
@@ -10580,7 +10583,7 @@
         <v>77</v>
       </c>
       <c r="W74" t="s" s="2">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="X74" t="s" s="2">
         <v>77</v>
@@ -10607,7 +10610,7 @@
         <v>77</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>78</v>
@@ -10636,14 +10639,14 @@
     </row>
     <row r="75" hidden="true">
       <c r="A75" t="s" s="2">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E75" s="2"/>
       <c r="F75" t="s" s="2">
@@ -10665,10 +10668,10 @@
         <v>164</v>
       </c>
       <c r="L75" t="s" s="2">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="M75" t="s" s="2">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
@@ -10719,7 +10722,7 @@
         <v>77</v>
       </c>
       <c r="AF75" t="s" s="2">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>78</v>
@@ -10734,13 +10737,13 @@
         <v>99</v>
       </c>
       <c r="AK75" t="s" s="2">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="AL75" t="s" s="2">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="AM75" t="s" s="2">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="AN75" t="s" s="2">
         <v>77</v>
@@ -10748,14 +10751,14 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E76" s="2"/>
       <c r="F76" t="s" s="2">
@@ -10777,10 +10780,10 @@
         <v>164</v>
       </c>
       <c r="L76" t="s" s="2">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="M76" t="s" s="2">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="N76" s="2"/>
       <c r="O76" s="2"/>
@@ -10795,7 +10798,7 @@
         <v>77</v>
       </c>
       <c r="T76" t="s" s="2">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="U76" t="s" s="2">
         <v>77</v>
@@ -10831,7 +10834,7 @@
         <v>77</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>78</v>
@@ -10846,13 +10849,13 @@
         <v>99</v>
       </c>
       <c r="AK76" t="s" s="2">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="AL76" t="s" s="2">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="AM76" t="s" s="2">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="AN76" t="s" s="2">
         <v>77</v>
@@ -10860,10 +10863,10 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -10889,13 +10892,13 @@
         <v>164</v>
       </c>
       <c r="L77" t="s" s="2">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="M77" t="s" s="2">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="N77" t="s" s="2">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="O77" s="2"/>
       <c r="P77" t="s" s="2">
@@ -10945,7 +10948,7 @@
         <v>77</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>78</v>
@@ -10960,13 +10963,13 @@
         <v>99</v>
       </c>
       <c r="AK77" t="s" s="2">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="AL77" t="s" s="2">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="AM77" t="s" s="2">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="AN77" t="s" s="2">
         <v>77</v>
@@ -10974,10 +10977,10 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -11003,14 +11006,14 @@
         <v>222</v>
       </c>
       <c r="L78" t="s" s="2">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="M78" t="s" s="2">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="N78" s="2"/>
       <c r="O78" t="s" s="2">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="P78" t="s" s="2">
         <v>77</v>
@@ -11023,7 +11026,7 @@
         <v>77</v>
       </c>
       <c r="T78" t="s" s="2">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="U78" t="s" s="2">
         <v>77</v>
@@ -11059,7 +11062,7 @@
         <v>77</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>78</v>
@@ -11074,10 +11077,10 @@
         <v>99</v>
       </c>
       <c r="AK78" t="s" s="2">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="AL78" t="s" s="2">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="AM78" t="s" s="2">
         <v>228</v>
@@ -11088,10 +11091,10 @@
     </row>
     <row r="79">
       <c r="A79" t="s" s="2">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -11114,17 +11117,17 @@
         <v>88</v>
       </c>
       <c r="K79" t="s" s="2">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="L79" t="s" s="2">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="M79" t="s" s="2">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="N79" s="2"/>
       <c r="O79" t="s" s="2">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="P79" t="s" s="2">
         <v>77</v>
@@ -11173,7 +11176,7 @@
         <v>77</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>78</v>
@@ -11191,7 +11194,7 @@
         <v>259</v>
       </c>
       <c r="AL79" t="s" s="2">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="AM79" t="s" s="2">
         <v>168</v>
@@ -11202,10 +11205,10 @@
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -11228,19 +11231,19 @@
         <v>77</v>
       </c>
       <c r="K80" t="s" s="2">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="L80" t="s" s="2">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="M80" t="s" s="2">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="N80" t="s" s="2">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="O80" t="s" s="2">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="P80" t="s" s="2">
         <v>77</v>
@@ -11289,7 +11292,7 @@
         <v>77</v>
       </c>
       <c r="AF80" t="s" s="2">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="AG80" t="s" s="2">
         <v>78</v>
@@ -11307,7 +11310,7 @@
         <v>77</v>
       </c>
       <c r="AL80" t="s" s="2">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="AM80" t="s" s="2">
         <v>77</v>
@@ -11318,10 +11321,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -11430,10 +11433,10 @@
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -11544,14 +11547,14 @@
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E83" s="2"/>
       <c r="F83" t="s" s="2">
@@ -11573,10 +11576,10 @@
         <v>133</v>
       </c>
       <c r="L83" t="s" s="2">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="M83" t="s" s="2">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="N83" t="s" s="2">
         <v>136</v>
@@ -11631,7 +11634,7 @@
         <v>77</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>78</v>
@@ -11660,10 +11663,10 @@
     </row>
     <row r="84" hidden="true">
       <c r="A84" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -11689,14 +11692,14 @@
         <v>188</v>
       </c>
       <c r="L84" t="s" s="2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="M84" t="s" s="2">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="N84" s="2"/>
       <c r="O84" t="s" s="2">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="P84" t="s" s="2">
         <v>77</v>
@@ -11724,10 +11727,10 @@
         <v>193</v>
       </c>
       <c r="Y84" t="s" s="2">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="Z84" t="s" s="2">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="AA84" t="s" s="2">
         <v>77</v>
@@ -11745,7 +11748,7 @@
         <v>77</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>78</v>
@@ -11763,7 +11766,7 @@
         <v>77</v>
       </c>
       <c r="AL84" t="s" s="2">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="AM84" t="s" s="2">
         <v>77</v>
@@ -11774,10 +11777,10 @@
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -11800,17 +11803,17 @@
         <v>77</v>
       </c>
       <c r="K85" t="s" s="2">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="L85" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="M85" t="s" s="2">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="N85" s="2"/>
       <c r="O85" t="s" s="2">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="P85" t="s" s="2">
         <v>77</v>
@@ -11859,7 +11862,7 @@
         <v>77</v>
       </c>
       <c r="AF85" t="s" s="2">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="AG85" t="s" s="2">
         <v>78</v>
@@ -11874,10 +11877,10 @@
         <v>99</v>
       </c>
       <c r="AK85" t="s" s="2">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="AL85" t="s" s="2">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="AM85" t="s" s="2">
         <v>77</v>
@@ -11888,10 +11891,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -11914,17 +11917,17 @@
         <v>77</v>
       </c>
       <c r="K86" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="L86" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="M86" t="s" s="2">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="N86" s="2"/>
       <c r="O86" t="s" s="2">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="P86" t="s" s="2">
         <v>77</v>
@@ -11973,7 +11976,7 @@
         <v>77</v>
       </c>
       <c r="AF86" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>78</v>
@@ -11988,10 +11991,10 @@
         <v>99</v>
       </c>
       <c r="AK86" t="s" s="2">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="AL86" t="s" s="2">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="AM86" t="s" s="2">
         <v>77</v>
@@ -12002,10 +12005,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -12028,17 +12031,17 @@
         <v>77</v>
       </c>
       <c r="K87" t="s" s="2">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="L87" t="s" s="2">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="M87" t="s" s="2">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="N87" s="2"/>
       <c r="O87" t="s" s="2">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="P87" t="s" s="2">
         <v>77</v>
@@ -12087,7 +12090,7 @@
         <v>77</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>78</v>
@@ -12102,10 +12105,10 @@
         <v>99</v>
       </c>
       <c r="AK87" t="s" s="2">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="AL87" t="s" s="2">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="AM87" t="s" s="2">
         <v>77</v>
@@ -12116,10 +12119,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -12142,17 +12145,17 @@
         <v>77</v>
       </c>
       <c r="K88" t="s" s="2">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="L88" t="s" s="2">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="M88" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="N88" s="2"/>
       <c r="O88" t="s" s="2">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="P88" t="s" s="2">
         <v>77</v>
@@ -12201,7 +12204,7 @@
         <v>77</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>78</v>

</xml_diff>